<commit_message>
Add detailed component sourcing guide for SA32 project in součástky.txt
- Included a comprehensive list of key Czech and EU online shops for sourcing components.
- Provided real prices and availability for each component in the BOM.
- Suggested alternatives and highlighted potential issues with specific components.
- Offered a recalculated total cost based on real prices and shopping strategies.
</commit_message>
<xml_diff>
--- a/docs/SA32_BOM.xlsx
+++ b/docs/SA32_BOM.xlsx
@@ -7,9 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="BOM" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="GPIO map" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Napájení" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="BOM v1.1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="GPIO map v1.1" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Napájení v1.1" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Validace HW" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,10 +33,27 @@
       <color rgb="00FFFFFF"/>
     </font>
     <font>
+      <color rgb="001D4ED8"/>
+      <sz val="9"/>
+      <u val="single"/>
+    </font>
+    <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00047857"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00B45309"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001D4ED8"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -45,6 +63,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="000D9488"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF3C7"/>
       </patternFill>
     </fill>
     <fill>
@@ -84,7 +107,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -92,13 +115,34 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -465,18 +509,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:K28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="4" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
     <col width="38" customWidth="1" min="6" max="6"/>
-    <col width="36" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -512,17 +558,27 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Dodavatelé (CZ/EU)</t>
+          <t>E-shop</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>Cena/ks (CZK)</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Cena celkem (CZK)</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>v1.1</t>
         </is>
       </c>
     </row>
@@ -545,25 +601,31 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>ESP32-S3-DevKitC-1 (WROOM-1-N16R8, 16 MB flash, 8 MB octal PSRAM)</t>
+          <t>ESP32-S3-DevKitC-1 N16R8 (16 MB flash, 8 MB octal PSRAM)</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>DevKit modul, USB-C</t>
+          <t>DevKit modul s USB-C; ⚠ ověř N16R8 variantu, ne N8R8</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Mouser.cz, DigiKey.cz, LaskaKit.cz, PUHY.cz</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="n">
-        <v>650</v>
+          <t>Allegro.cz / LaskaKit</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>otevřít</t>
+        </is>
       </c>
       <c r="I2" s="2" t="n">
-        <v>650</v>
-      </c>
+        <v>316</v>
+      </c>
+      <c r="J2" s="2" t="n">
+        <v>316</v>
+      </c>
+      <c r="K2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -584,25 +646,31 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>PCM5102A I²S DAC breakout (SCK→GND, line out 2.1 Vrms)</t>
+          <t>PCM5102A I²S DAC modul (GY-PCM5102, line-out 2,1 Vrms)</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>modul ~38×25 mm</t>
+          <t>modul ~38×25 mm, SCK→GND interní PLL</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>LaskaKit.cz, TinyTronics.nl, AliExpress EU</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="n">
-        <v>220</v>
+          <t>LaskaKit</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>otevřít</t>
+        </is>
       </c>
       <c r="I3" s="2" t="n">
-        <v>220</v>
-      </c>
+        <v>130</v>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>130</v>
+      </c>
+      <c r="K3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -623,102 +691,128 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>TPA3110D2 2×15 W class-D zesilovač modul</t>
+          <t>TPA3110D2 2×15 W class-D modul (XH-A232)</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>PBTL/stereo DIP zkratovací, 12–24 V vstup</t>
+          <t>PBTL/stereo jumper, VIN 12–24 V; ⚠ nastav GAIN=12 dB jumperem</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>AliExpress EU, GM Electronic</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="n">
-        <v>220</v>
+          <t>Hadex</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>otevřít</t>
+        </is>
       </c>
       <c r="I4" s="2" t="n">
-        <v>220</v>
-      </c>
+        <v>120</v>
+      </c>
+      <c r="J4" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="K4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Audio</t>
         </is>
       </c>
-      <c r="C5" s="2" t="n">
+      <c r="C5" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>J1</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Stereo 3.5 mm jack PCB (vstup z DAC do AMP)</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>stíněný kablík ~10 cm</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>GM Electronic, TME.eu</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="n">
-        <v>35</v>
-      </c>
-      <c r="I5" s="2" t="n">
-        <v>35</v>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>U7</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>BK3266 / BLK-MD-SPK Bluetooth receiver s I²S výstupem</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>BT 5.0 BR/EDR, A2DP/AVRCP přes UART AT příkazy, 3,3 V napájení</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>Allegro.cz</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>otevřít</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="n">
+        <v>130</v>
+      </c>
+      <c r="J5" s="4" t="n">
+        <v>130</v>
+      </c>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>UI</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="n">
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Audio</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>U4</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>OLED displej SSD1306 128×64 I²C, adresa 0x3C, 0,96"</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>VCC 3,3 V, 4-pin (SDA/SCL/VCC/GND)</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>Robotstore.cz, Pajtech.cz, LaskaKit.cz</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="n">
-        <v>130</v>
-      </c>
-      <c r="I6" s="2" t="n">
-        <v>130</v>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>U8</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>I²S MUX NX3L4684 (3-kanál 2:1, R_on 0,5 Ω)</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>TSSOP-14; alt. 74HC4053 v DIP-16 (8 Kč) pro DIY</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>TME.cz</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>otevřít</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -727,7 +821,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Audio</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
@@ -735,30 +829,36 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>S1</t>
+          <t>J1</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Rotační enkodér Alps EC11 (24 pulzů, taktilní switch)</t>
+          <t>Stereo 3,5 mm jack PCB pro propojení DAC → AMP</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>vyveden A/B/SW + 2× GND, hřídel 20 mm</t>
+          <t>stíněný kablík ~10 cm, stínění zem jen na DAC straně</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Mouser.cz, Farnell.cz, TME.eu</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="n">
-        <v>75</v>
+          <t>GME</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>otevřít</t>
+        </is>
       </c>
       <c r="I7" s="2" t="n">
-        <v>75</v>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="J7" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="K7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -774,30 +874,36 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>K1</t>
+          <t>U4</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Knoflík hliníkový 6 mm D-shaft, ⌀ 20 mm</t>
+          <t>OLED displej SSD1306 / SSD1315 0,96" 128×64 I²C</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>matný hliník</t>
+          <t>I²C 0x3C, napájení 3,3 V (NIKDY ne 5 V), pull-upy onboard</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>TME.eu, Mouser.cz</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="n">
-        <v>60</v>
+          <t>LaskaKit</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>otevřít</t>
+        </is>
       </c>
       <c r="I8" s="2" t="n">
-        <v>60</v>
-      </c>
+        <v>100</v>
+      </c>
+      <c r="J8" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="K8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -805,7 +911,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Power</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
@@ -813,30 +919,36 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>PSU</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Mean Well IRM-20-24 (24 V / 20 W) nebo ekvivalent</t>
+          <t>Rotační enkodér Alps EC11 (24 pulzů, taktilní switch)</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>AC/DC zalitý modul</t>
+          <t>vyveden A/B/SW + 2× GND; alt. 20-pulzní za 41 Kč na Allegru</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>GM Electronic (gme.cz), Mouser.cz</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="n">
-        <v>350</v>
+          <t>TME.cz</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>otevřít</t>
+        </is>
       </c>
       <c r="I9" s="2" t="n">
-        <v>350</v>
-      </c>
+        <v>70</v>
+      </c>
+      <c r="J9" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="K9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -844,7 +956,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Power</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
@@ -852,146 +964,182 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>J2</t>
+          <t>K1</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Souosý DC jack 5,5/2,1 mm panelový</t>
+          <t>Hliníkový knoflík ⌀20 mm, D-shaft 6 mm</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>lepený / matka</t>
+          <t>matný hliník, hřídel 20 mm</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>GME, TME.eu</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="n">
-        <v>30</v>
+          <t>TME.cz</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>otevřít</t>
+        </is>
       </c>
       <c r="I10" s="2" t="n">
-        <v>30</v>
-      </c>
+        <v>60</v>
+      </c>
+      <c r="J10" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="K10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n">
+      <c r="A11" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>Power</t>
         </is>
       </c>
-      <c r="C11" s="2" t="n">
+      <c r="C11" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>U5</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>AMS1117-3.3 LDO modul (vstup 5 V → 3,3 V, ≥ 500 mA)</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>alt: napájení z USB DevKitu při dev</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>GME, LaskaKit.cz</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="n">
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>PSU</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Mean Well IRM-45-24 (24 V / 1,88 A / 45 W, AC/DC zalitý modul)</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>drop-in upgrade z IRM-20-24, +30 % rezerva nad 1,44 A peak AMP</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>GME</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>otevřít</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="n">
+        <v>490</v>
+      </c>
+      <c r="J11" s="4" t="n">
+        <v>490</v>
+      </c>
+      <c r="K11" s="4" t="inlineStr">
+        <is>
+          <t>UPGRADE</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Power</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>U6</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>HLK-5M05 izolovaný buck 24 V → 5 V / 1 A (5 W)</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>primárně izolovaný = bez ground loopu; alt. MP1584 (45 Kč) ale rušivý</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>GME</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>otevřít</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="n">
+        <v>90</v>
+      </c>
+      <c r="J12" s="4" t="n">
+        <v>90</v>
+      </c>
+      <c r="K12" s="4" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Power</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>U9</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>AMS1117-3.3 / AP2112K-3.3 modul nebo SOT-223 + caps</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>5 V → 3,3 V LDO pro DAC + OLED (~30 mA), uvolní DevKit AMS1117</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>GME</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>otevřít</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="I11" s="2" t="n">
+      <c r="J13" s="4" t="n">
         <v>25</v>
       </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Power</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>U6</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>AP2112-1.8 LDO (volitelné, čistá analogová větev DAC)</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>SOT-23-5</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>Mouser.cz, Farnell.cz</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="I12" s="2" t="n">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>Power</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>Tavná pojistka 5×20 mm 1,6 A T + držák</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>primární strana 230 V</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>GME, TME.eu</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="n">
-        <v>35</v>
-      </c>
-      <c r="I13" s="2" t="n">
-        <v>35</v>
+      <c r="K13" s="4" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -1000,38 +1148,44 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Passive</t>
+          <t>Power</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>C1,C2</t>
+          <t>F1</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Elektrolyt 1000 µF / 35 V low-ESR</t>
+          <t>Pojistka 5×20 mm 1,6 A T (slow-blow) + držák do panelu</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>filtrace 24 V vstupu AMP</t>
+          <t>primární strana 230 V — POVINNÉ pro bezpečnost</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>GME, TME.eu</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="n">
-        <v>25</v>
+          <t>GME</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>otevřít</t>
+        </is>
       </c>
       <c r="I14" s="2" t="n">
-        <v>50</v>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="J14" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="K14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -1039,38 +1193,44 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Passive</t>
+          <t>Power</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>C3,C4</t>
+          <t>J2</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>MLCC 100 nF / 50 V X7R 0,1"</t>
+          <t>DC jack 5,5 / 2,1 mm panelový (pro IRM-45-24 výstup)</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>blok napájení</t>
+          <t>nebo přímý drát z IRM do AMP (úspora 30 Kč, mínus modularita)</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>GME, TME.eu</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="n">
-        <v>3</v>
+          <t>GME</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>otevřít</t>
+        </is>
       </c>
       <c r="I15" s="2" t="n">
-        <v>6</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="J15" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="K15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -1086,17 +1246,17 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>R1,R2</t>
+          <t>C1, C2</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Pull-up 10 kΩ 1/4 W (rezerva pro I²C, pokud modul nemá)</t>
+          <t>Elektrolyt 1000 µF / 35 V low-ESR</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>většina OLED breakoutů má vlastní</t>
+          <t>filtrace 24 V vstupu AMP; doporučeno Panasonic FM serie</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -1104,12 +1264,18 @@
           <t>GME</t>
         </is>
       </c>
-      <c r="H16" s="2" t="n">
-        <v>2</v>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>otevřít</t>
+        </is>
       </c>
       <c r="I16" s="2" t="n">
-        <v>4</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="J16" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="K16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -1121,111 +1287,137 @@
         </is>
       </c>
       <c r="C17" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>C3-C6</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>MLCC 100 nF / 50 V X7R</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>blok napájení každého aktivního IC (DAC, MUX, BT, LDO)</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>GME</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>otevřít</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="J17" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="K17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>R3,R4</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>Sériový rezistor 33 Ω I²C (volitelně, ringing fix)</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>v případě dlouhého wiringu</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>C7, C8</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>MLCC 47 µF / 16 V X5R</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>Pi filtr na 5 V výstupu HLK-5M05 (před a za ferrit beadem)</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
         <is>
           <t>GME</t>
         </is>
       </c>
-      <c r="H17" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="I17" s="2" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Mech</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>Reproduktor 8 Ω / ≥ 15 W (3–4" full-range)</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>podle krabičky</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>Reichelt.cz, TME.eu</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="n">
-        <v>280</v>
-      </c>
-      <c r="I18" s="2" t="n">
-        <v>560</v>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>otevřít</t>
+        </is>
+      </c>
+      <c r="I18" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="J18" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="K18" s="4" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="n">
+      <c r="A19" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>Mech</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="n">
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>BOX</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>Hliníková krabička ~120×100×45 mm (např. Hammond 1455)</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>frézování čela pro OLED + enkodér</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>TME.eu, Mouser.cz</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="n">
-        <v>320</v>
-      </c>
-      <c r="I19" s="2" t="n">
-        <v>320</v>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Ferritový bead BLM31KN601SN1 (600 Ω @ 100 MHz, 0805/1206)</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>v sérii s 5 V z buck před AMS1117 — potlačí spínací harmonické</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>GME</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>otevřít</t>
+        </is>
+      </c>
+      <c r="I19" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J19" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="K19" s="4" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -1234,38 +1426,44 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Mech</t>
+          <t>Passive</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>WIRE</t>
+          <t>R1-R4</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Sada propojovacích vodičů Dupont F-F + silnější 18 AWG (PSU/SPK)</t>
+          <t>Sada rezistorů (4,7 kΩ pull-up, 33 Ω I²C série, 470 Ω LED)</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>mix</t>
+          <t>1/4 W, 5 %; pokud máš sadu 600+ ks, použij ji</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>GME, AliExpress</t>
-        </is>
-      </c>
-      <c r="H20" s="2" t="n">
-        <v>80</v>
+          <t>GME</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>otevřít</t>
+        </is>
       </c>
       <c r="I20" s="2" t="n">
-        <v>80</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="J20" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="K20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -1277,124 +1475,304 @@
         </is>
       </c>
       <c r="C21" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Reproduktor 8 Ω / ≥ 15 W, 3–4" full-range</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>podle krabičky a poslechu; alternativa 2-pásmový mini-monitor</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>TME.cz</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>otevřít</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="n">
+        <v>280</v>
+      </c>
+      <c r="J21" s="2" t="n">
+        <v>560</v>
+      </c>
+      <c r="K21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Mech</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>BOX</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Hliníková krabička Hammond 1455N1601 (~120×100×45 mm)</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>frézování čela pro OLED + enkodér; alt. levnější ABS box ~200 Kč</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>TME.cz</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>otevřít</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="n">
+        <v>450</v>
+      </c>
+      <c r="J22" s="2" t="n">
+        <v>450</v>
+      </c>
+      <c r="K22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Mech</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>WIRE</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Sada propojovacích vodičů Dupont F-F + silnější 18 AWG</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>mix barev pro snadnou orientaci</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>GME</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>otevřít</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="J23" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="K23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Mech</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>STAND</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>Stojánky M3 mosaz 8 mm + šrouby/matky (4 ks DAC, 4 ks AMP, 4 ks DevKit)</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>izolace od šasi</t>
-        </is>
-      </c>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t>GME, TME.eu</t>
-        </is>
-      </c>
-      <c r="H21" s="2" t="n">
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Distanční sloupky M3 mosaz 8 mm + šrouby/matky</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>izolace modulů od šasi, sada ~20 ks</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>GME</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>otevřít</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="I21" s="2" t="n">
+      <c r="J24" s="2" t="n">
         <v>45</v>
       </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="n">
-        <v>21</v>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="K24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
       </c>
-      <c r="C22" s="3" t="n">
+      <c r="C25" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>LED1, LED2</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>Status LED 3 mm + 470 Ω (Wi-Fi / BT indikace na GPIO 38/39)</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>Kconfig SOKOL_STATUS_LEDS_ENABLE</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>GME</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>otevřít</t>
+        </is>
+      </c>
+      <c r="I25" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="J25" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="K25" s="6" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>U7</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr">
-        <is>
-          <t>PCM5102A XSMT vyvedení (digi mute) — pokud modul má pad</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>GPIO13, Kconfig SOKOL_DAC_MUTE_PIN_ENABLE</t>
-        </is>
-      </c>
-      <c r="G22" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H22" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I22" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="n">
-        <v>22</v>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>LED</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="inlineStr">
-        <is>
-          <t>Status LED 3 mm + 470 Ω (WiFi/BT) — GPIO38/39</t>
-        </is>
-      </c>
-      <c r="F23" s="3" t="inlineStr">
-        <is>
-          <t>Kconfig SOKOL_STATUS_LEDS_ENABLE</t>
-        </is>
-      </c>
-      <c r="G23" s="3" t="inlineStr">
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>U10</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>Krátký USB-C kabel pro flashování + sériovou konzoli</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>USB-C k DevKitu, 0,5 m stačí</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr">
         <is>
           <t>GME</t>
         </is>
       </c>
-      <c r="H23" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="I23" s="3" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="H25" s="4" t="inlineStr">
-        <is>
-          <t>CELKEM (orient.)</t>
-        </is>
-      </c>
-      <c r="I25" s="5" t="n">
-        <v>2940</v>
+      <c r="H26" s="7" t="inlineStr">
+        <is>
+          <t>otevřít</t>
+        </is>
+      </c>
+      <c r="I26" s="6" t="n">
+        <v>90</v>
+      </c>
+      <c r="J26" s="6" t="n">
+        <v>90</v>
+      </c>
+      <c r="K26" s="6" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="I28" s="8" t="inlineStr">
+        <is>
+          <t>CELKEM (povinné, orient.)</t>
+        </is>
+      </c>
+      <c r="J28" s="9" t="n">
+        <v>2887</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId25"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1405,7 +1783,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1417,32 +1795,32 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>GPIO</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="10" t="inlineStr">
         <is>
           <t>Funkce</t>
         </is>
       </c>
-      <c r="C1" s="6" t="inlineStr">
+      <c r="C1" s="10" t="inlineStr">
         <is>
           <t>Směr</t>
         </is>
       </c>
-      <c r="D1" s="6" t="inlineStr">
+      <c r="D1" s="10" t="inlineStr">
         <is>
           <t>Pull / IRQ</t>
         </is>
       </c>
-      <c r="E1" s="6" t="inlineStr">
+      <c r="E1" s="10" t="inlineStr">
         <is>
           <t>Připojení</t>
         </is>
       </c>
-      <c r="F1" s="6" t="inlineStr">
+      <c r="F1" s="10" t="inlineStr">
         <is>
           <t>Pozn.</t>
         </is>
@@ -1469,12 +1847,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>PCM5102A BCK</t>
+          <t>MUX → PCM5102A BCK</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>44,1 kHz × 32 = 1,4112 MHz</t>
+          <t>1,4112 MHz @ 44,1 kHz S16</t>
         </is>
       </c>
     </row>
@@ -1499,12 +1877,12 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>PCM5102A LCK</t>
+          <t>MUX → PCM5102A LCK</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>WS, 44,1 kHz</t>
+          <t>44,1 kHz word select</t>
         </is>
       </c>
     </row>
@@ -1529,12 +1907,12 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>PCM5102A DIN</t>
+          <t>MUX → PCM5102A DIN</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>S16LE stereo</t>
+          <t>stereo S16LE</t>
         </is>
       </c>
     </row>
@@ -1584,7 +1962,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>pull-up int.</t>
+          <t>PU int.</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -1594,7 +1972,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>400 kHz, sdílí budoucí I²C</t>
+          <t>400 kHz</t>
         </is>
       </c>
     </row>
@@ -1614,7 +1992,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>pull-up int.</t>
+          <t>PU int.</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -1740,7 +2118,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>active HIGH = ticho, default při bootu</t>
+          <t>active HIGH = ticho, default boot</t>
         </is>
       </c>
     </row>
@@ -1775,60 +2153,180 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="n">
+      <c r="A13" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>I²S MUX SEL</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>out</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>PD external</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>NX3L4684 SEL</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>v1.1 NEW: 0=ESP, 1=BT</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>BK3266 RESET</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>out</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>BK3266 nReset</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>v1.1 NEW: active LOW pulse</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>UART2 TX</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>out</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>BK3266 RX</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>v1.1 NEW: AT příkazy 115200</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>UART2 RX</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>BK3266 TX</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>v1.1 NEW: status events</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
         <v>38</v>
       </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>WiFi LED (opt)</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Wi-Fi LED (opt)</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>out</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>LED → 470 Ω → GND</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>Kconfig SOKOL_STATUS_LEDS_ENABLE</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="n">
+    <row r="18">
+      <c r="A18" s="2" t="n">
         <v>39</v>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>BT LED (opt)</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>out</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>LED → 470 Ω → GND</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1841,47 +2339,53 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>Větev</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="10" t="inlineStr">
         <is>
           <t>Napětí</t>
         </is>
       </c>
-      <c r="C1" s="6" t="inlineStr">
+      <c r="C1" s="10" t="inlineStr">
         <is>
           <t>Typický odběr</t>
         </is>
       </c>
-      <c r="D1" s="6" t="inlineStr">
+      <c r="D1" s="10" t="inlineStr">
         <is>
           <t>Špička</t>
         </is>
       </c>
-      <c r="E1" s="6" t="inlineStr">
+      <c r="E1" s="10" t="inlineStr">
         <is>
           <t>Zdroj</t>
+        </is>
+      </c>
+      <c r="F1" s="10" t="inlineStr">
+        <is>
+          <t>Ztráta</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>AMP (TPA3110D2)</t>
+          <t>AMP TPA3110D2 (2×15 W RMS)</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -1891,78 +2395,93 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>150 mA (klid)</t>
+          <t>150 mA klid</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>1,2 A (15 W RMS)</t>
+          <t>1,44 A peak</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>IRM-20-24</t>
+          <t>IRM-45-24 (1,88 A) — 30 % rezerva</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>4,5 W na čipu (heatsink)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>ESP32-S3 DevKit</t>
+          <t>Logic 5 V (přes HLK-5M05)</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>5 V</t>
+          <t>24 V</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>120 mA</t>
+          <t>0,2 A vstup</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>350 mA (BT TX)</t>
+          <t>0,5 A vstup</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>USB během vývoje, jinak 5 V z PSU větve</t>
+          <t>IRM-45-24 stejný rail</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>0,33 W v HLK</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>ESP32-S3 jádro</t>
+          <t>DevKit ESP32-S3 (přes onb. AMS1117)</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>3,3 V</t>
+          <t>5 V</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>120 mA</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>500 mA Wi-Fi TX</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>interní LDO DevKitu</t>
+          <t>HLK-5M05</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>0,93 W na DevKit AMS</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>PCM5102A DAC</t>
+          <t>BK3266 BT receiver</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -1972,24 +2491,29 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>20 mA</t>
+          <t>35 mA</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>30 mA</t>
+          <t>50 mA streaming</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>AMS1117-3.3 (sdílí s ESP)</t>
+          <t>externí AMS1117 (U9) z 5 V</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>&lt;0,1 W</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>SSD1306 OLED</t>
+          <t>PCM5102A DAC</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -1999,24 +2523,29 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>8 mA</t>
+          <t>20 mA</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>20 mA (vše svítí)</t>
+          <t>30 mA</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>AMS1117-3.3</t>
+          <t>externí AMS1117 (U9) z 5 V</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>&lt;0,1 W</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>EC11 enkodér</t>
+          <t>SSD1306 OLED</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -2026,44 +2555,541 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>&lt; 1 mA</t>
+          <t>8 mA</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>20 mA</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>interní pull-upy</t>
+          <t>externí AMS1117 (U9) z 5 V</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>&lt;0,1 W</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Reproduktory</t>
+          <t>EC11 enkodér</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
+          <t>3,3 V</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>&lt; 1 mA</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>interní pull-upy ESP32</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>&lt;0,01 W</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>NX3L4684 MUX</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>3,3 V</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>&lt; 1 mA</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>10 mA</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>externí AMS1117 (U9) z 5 V</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>&lt;0,01 W</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Reproduktory 2× 8 Ω</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>2× 15 W RMS</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>BTL z TPA3110D2</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="10" t="inlineStr">
+        <is>
+          <t>Kontrola</t>
+        </is>
+      </c>
+      <c r="C1" s="10" t="inlineStr">
+        <is>
+          <t>Spec / norma</t>
+        </is>
+      </c>
+      <c r="D1" s="10" t="inlineStr">
+        <is>
+          <t>Výsledek</t>
+        </is>
+      </c>
+      <c r="E1" s="10" t="inlineStr">
+        <is>
+          <t>Pozn.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>PSU nadproudová rezerva</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>I_max ≥ 1,3 × I_peak</t>
+        </is>
+      </c>
+      <c r="D2" s="11" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>1,88 A / 1,44 A = 130 %</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>5 V buck výkonová rezerva</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>P_max ≥ 1,5 × P_avg</t>
+        </is>
+      </c>
+      <c r="D3" s="11" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>5 W / 2,8 W = 178 %</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>AMS1117 termální (DevKit)</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>P_diss &lt; 1 W bez heatsinku</t>
+        </is>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>BORDERLINE</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>0,93 W peak — odlehčit ext. LDO</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>I²S BCLK přes MUX</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>f_max NX3L4684 &gt; 1,4 MHz</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>NX3L4684 propustnost &gt; 100 MHz</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Logické úrovně I²S</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>V_OH ≥ 2,0 V (V_IH PCM5102A)</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>ESP/BT 3,0 V min, DAC 2,0 V</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>DAC → AMP voltage match</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>V_in ≤ 1 Vrms při GAIN 20 dB</t>
+        </is>
+      </c>
+      <c r="D7" s="12" t="inlineStr">
+        <is>
+          <t>ACTION</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Nastavit GAIN jumper na 12 dB</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Pojistka primár</t>
+        </is>
+      </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>2× 15 W RMS</t>
+          <t>I_t = 1,6 A T pro 45 W zdroj</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>z TPA3110D2</t>
+          <t>F1 v sérii s L 230 V</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>BK3266 baud rate</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>115200 default firmware</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>potvrzeno pro většinu klonů</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Partition table OTA</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>2× ota_X (2 MB) + factory</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>partitions.csv beze změny</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Disable BR/EDR (ESP32-S3)</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>ESP_BT_ENABLED=n</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>úspora ~80 KB internal RAM</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>GPIO konflikty</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>žádné s octal PSRAM 35-37</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>MUX_SEL 4, BK_RST 14, UART2 17/18</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Audio cable shield</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>ground only at DAC end</t>
+        </is>
+      </c>
+      <c r="D13" s="13" t="inlineStr">
+        <is>
+          <t>DOC</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>v PDF zmíněno, vizuální kontrola</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Star ground topologie</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>single junction at PSU GND</t>
+        </is>
+      </c>
+      <c r="D14" s="13" t="inlineStr">
+        <is>
+          <t>DOC</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>manuál instaluje uživatel</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>OTA rollback</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>BOOTLOADER_APP_ROLLBACK_ENABLE</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>auto-validate po 30 s běhu</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>HTTPS cert verify</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>MBEDTLS_CERTIFICATE_BUNDLE</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>mozilla CA bundle</t>
         </is>
       </c>
     </row>

</xml_diff>